<commit_message>
Added new methods to NPS class
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_nps.xlsx
+++ b/BharatFinTrack/base_data/base_nps.xlsx
@@ -256,36 +256,36 @@
     <t>NPS TRUST - A/C UTI NPS SANCHAY SCHEME DIRECT</t>
   </si>
   <si>
+    <t>LIC PENSION FUND SCHEME - CENTRAL GOVT</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME - STATE GOVT</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C-LIC PENSION FUND LIMITED- NPS LITE SCHEME - GOVT. PATTERN</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND LIMITED SCHEME - CORPORATE-CG</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME E - TIER I</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME C - TIER I</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME G - TIER I</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME E - TIER II</t>
+  </si>
+  <si>
+    <t>LIC PENSION FUND SCHEME C - TIER II</t>
+  </si>
+  <si>
     <t>LIC PENSION FUND SCHEME G - TIER II</t>
   </si>
   <si>
-    <t>LIC PENSION FUND SCHEME - CENTRAL GOVT</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME - STATE GOVT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C-LIC PENSION FUND LIMITED- NPS LITE SCHEME - GOVT. PATTERN</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND LIMITED SCHEME - CORPORATE-CG</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME E - TIER I</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME C - TIER I</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME G - TIER I</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME E - TIER II</t>
-  </si>
-  <si>
-    <t>LIC PENSION FUND SCHEME C - TIER II</t>
-  </si>
-  <si>
     <t>NPS TRUST - A/C LIC PENSION FUND SCHEME - ATAL PENSION YOJANA (APY)</t>
   </si>
   <si>
@@ -1042,34 +1042,34 @@
     <t>SM002036</t>
   </si>
   <si>
+    <t>SM003001</t>
+  </si>
+  <si>
+    <t>SM003002</t>
+  </si>
+  <si>
+    <t>SM003003</t>
+  </si>
+  <si>
+    <t>SM003004</t>
+  </si>
+  <si>
+    <t>SM003005</t>
+  </si>
+  <si>
+    <t>SM003006</t>
+  </si>
+  <si>
+    <t>SM003007</t>
+  </si>
+  <si>
+    <t>SM003008</t>
+  </si>
+  <si>
+    <t>SM003009</t>
+  </si>
+  <si>
     <t>SM003010</t>
-  </si>
-  <si>
-    <t>SM003001</t>
-  </si>
-  <si>
-    <t>SM003002</t>
-  </si>
-  <si>
-    <t>SM003003</t>
-  </si>
-  <si>
-    <t>SM003004</t>
-  </si>
-  <si>
-    <t>SM003005</t>
-  </si>
-  <si>
-    <t>SM003006</t>
-  </si>
-  <si>
-    <t>SM003007</t>
-  </si>
-  <si>
-    <t>SM003008</t>
-  </si>
-  <si>
-    <t>SM003009</t>
   </si>
   <si>
     <t>SM003011</t>

</xml_diff>

<commit_message>
Added new methods in NPS class
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_nps.xlsx
+++ b/BharatFinTrack/base_data/base_nps.xlsx
@@ -640,60 +640,60 @@
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME E - TIER I</t>
   </si>
   <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER I</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER I</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME A - TIER I</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME E - TIER II</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER II</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER II</t>
+  </si>
+  <si>
+    <t>TATA PENSION MANAGEMENT LIMITED TAX SAVER - TIER II</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - TATA PENSION FUND NPS SMART RETIREMENT FUND - TIER I</t>
+  </si>
+  <si>
+    <t>NPS TRUST - A/C TATA PENSION FUND - NPS VATSALYA SCHEME DIRECT</t>
+  </si>
+  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I GS</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I GS</t>
+  </si>
+  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I GS</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I GS</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME A - TIER I</t>
-  </si>
-  <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME E - TIER II</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER II DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER II</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER II DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER II</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER II DIRECT</t>
   </si>
   <si>
-    <t>TATA PENSION MANAGEMENT LIMITED TAX SAVER - TIER II</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - TATA PENSION FUND NPS SMART RETIREMENT FUND - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST - A/C TATA PENSION FUND - NPS VATSALYA SCHEME DIRECT</t>
-  </si>
-  <si>
     <t>NPS TRUST - A/C TATA PENSION FUND - NPS VATSALYA SCHEME POP</t>
   </si>
   <si>
@@ -1426,58 +1426,58 @@
     <t>SM011001</t>
   </si>
   <si>
+    <t>SM011002</t>
+  </si>
+  <si>
+    <t>SM011003</t>
+  </si>
+  <si>
+    <t>SM011004</t>
+  </si>
+  <si>
+    <t>SM011005</t>
+  </si>
+  <si>
+    <t>SM011006</t>
+  </si>
+  <si>
+    <t>SM011007</t>
+  </si>
+  <si>
+    <t>SM011008</t>
+  </si>
+  <si>
+    <t>SM011009</t>
+  </si>
+  <si>
+    <t>SM011010</t>
+  </si>
+  <si>
     <t>SM011011</t>
   </si>
   <si>
+    <t>SM011012</t>
+  </si>
+  <si>
+    <t>SM011013</t>
+  </si>
+  <si>
     <t>SM011014</t>
   </si>
   <si>
-    <t>SM011002</t>
-  </si>
-  <si>
-    <t>SM011012</t>
-  </si>
-  <si>
     <t>SM011015</t>
   </si>
   <si>
-    <t>SM011003</t>
-  </si>
-  <si>
-    <t>SM011013</t>
-  </si>
-  <si>
     <t>SM011016</t>
   </si>
   <si>
-    <t>SM011004</t>
-  </si>
-  <si>
-    <t>SM011005</t>
-  </si>
-  <si>
     <t>SM011017</t>
   </si>
   <si>
-    <t>SM011006</t>
-  </si>
-  <si>
     <t>SM011018</t>
   </si>
   <si>
-    <t>SM011007</t>
-  </si>
-  <si>
     <t>SM011019</t>
-  </si>
-  <si>
-    <t>SM011008</t>
-  </si>
-  <si>
-    <t>SM011009</t>
-  </si>
-  <si>
-    <t>SM011010</t>
   </si>
   <si>
     <t>SM011020</t>

</xml_diff>

<commit_message>
Modified documentation for NPS class
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_nps.xlsx
+++ b/BharatFinTrack/base_data/base_nps.xlsx
@@ -154,6 +154,9 @@
     <t>NPS TRUST - A/C SBI NPS SANCHAY SCHEME DIRECT</t>
   </si>
   <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND - NPS LITE SCHEME GOVT. PATTERN DIRECT</t>
+  </si>
+  <si>
     <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME- CENTRAL GOVT</t>
   </si>
   <si>
@@ -247,9 +250,6 @@
     <t>NPS TRUST - A/C UTI PENSION FUND - NPS VATSALYA SCHEME POP</t>
   </si>
   <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND - NPS LITE SCHEME GOVT. PATTERN DIRECT</t>
-  </si>
-  <si>
     <t>NPS TRUST - A/C UTI NPS SANCHAY SCHEME POP</t>
   </si>
   <si>
@@ -940,6 +940,9 @@
     <t>SM001034</t>
   </si>
   <si>
+    <t>SM002034</t>
+  </si>
+  <si>
     <t>SM002001</t>
   </si>
   <si>
@@ -1031,9 +1034,6 @@
   </si>
   <si>
     <t>SM002033</t>
-  </si>
-  <si>
-    <t>SM002034</t>
   </si>
   <si>
     <t>SM002035</t>

</xml_diff>

<commit_message>
Add new NPS scheme
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_nps.xlsx
+++ b/BharatFinTrack/base_data/base_nps.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="539">
   <si>
     <t>PFM</t>
   </si>
@@ -154,102 +154,102 @@
     <t>NPS TRUST - A/C SBI NPS SANCHAY SCHEME DIRECT</t>
   </si>
   <si>
+    <t>UTI RETIREMENT SOLUTIONS  SCHEME G - TIER II</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME- CENTRAL GOVT</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME- STATE GOVT</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME E - TIER I</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME C - TIER I</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME G - TIER I</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS SCHEME E - TIER II</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS SCHEME C - TIER II</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C-UTI RETIREMENT SOLUTIONS LIMITED- NPS LITE SCHEME - GOVT. PATTERN</t>
+  </si>
+  <si>
+    <t>NPS TRUST - A/C UTI RETIREMENT SOLUTIONS LTD. SCHEME - ATAL PENSION YOJANA (APY)</t>
+  </si>
+  <si>
+    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME A - TIER I</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C-UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME TAX SAVER TIER II</t>
+  </si>
+  <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME - APY FUND SCHEME</t>
+  </si>
+  <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME - NPS TIER- II COMPOSITE</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME - UPS CG SCHEME</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME - UPS POOL CG SCHEME</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PF WEALTH BUILDER NPS EQUITY SCHEME - TIER I</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PF WEALTH BUILDER NPS EQUITY SCHEME - TIER II</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PF DYNAMIC ASSET ALLOCATOR NPS SCHEME - TIER I</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PF DYNAMIC ASSET ALLOCATOR NPS SCHEME TIER II</t>
+  </si>
+  <si>
+    <t>NPS TRUST - A/C UTI PENSION FUND - NPS VATSALYA SCHEME DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME E - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME C - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME G - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME E - TIER I DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME C - TIER I DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME G - TIER I DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME E - TIER II DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME C - TIER II DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME G - TIER II DIRECT</t>
+  </si>
+  <si>
+    <t>NPS TRUST - A/C UTI PENSION FUND - NPS VATSALYA SCHEME POP</t>
+  </si>
+  <si>
     <t>NPS TRUST- A/C - UTI PENSION FUND - NPS LITE SCHEME GOVT. PATTERN DIRECT</t>
   </si>
   <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME- CENTRAL GOVT</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME- STATE GOVT</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME E - TIER I</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME C - TIER I</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME G - TIER I</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS SCHEME E - TIER II</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS SCHEME C - TIER II</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS  SCHEME G - TIER II</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C-UTI RETIREMENT SOLUTIONS LIMITED- NPS LITE SCHEME - GOVT. PATTERN</t>
-  </si>
-  <si>
-    <t>NPS TRUST - A/C UTI RETIREMENT SOLUTIONS LTD. SCHEME - ATAL PENSION YOJANA (APY)</t>
-  </si>
-  <si>
-    <t>UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME A - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C-UTI RETIREMENT SOLUTIONS PENSION FUND SCHEME TAX SAVER TIER II</t>
-  </si>
-  <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME - APY FUND SCHEME</t>
-  </si>
-  <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME - NPS TIER- II COMPOSITE</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME - UPS CG SCHEME</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME - UPS POOL CG SCHEME</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PF WEALTH BUILDER NPS EQUITY SCHEME - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PF WEALTH BUILDER NPS EQUITY SCHEME - TIER II</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PF DYNAMIC ASSET ALLOCATOR NPS SCHEME - TIER I</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PF DYNAMIC ASSET ALLOCATOR NPS SCHEME TIER II</t>
-  </si>
-  <si>
-    <t>NPS TRUST - A/C UTI PENSION FUND - NPS VATSALYA SCHEME DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME E - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME C - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME G - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME E - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME C - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C - UTI PENSION FUND SCHEME G - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME E - TIER II DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME C - TIER II DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST- A/C - UTI PENSION FUND SCHEME G - TIER II DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST - A/C UTI PENSION FUND - NPS VATSALYA SCHEME POP</t>
-  </si>
-  <si>
     <t>NPS TRUST - A/C UTI NPS SANCHAY SCHEME POP</t>
   </si>
   <si>
@@ -418,6 +418,9 @@
     <t>NPS TRUST - A/C KOTAK MAHINDRA PENSION FUND - NPS VATSALYA SCHEME POP</t>
   </si>
   <si>
+    <t>NPS TRUST A/C-KOTAK MAHINDRA PENSION FUND LIMITED- NPS LITE SCHEME - GOVT. PATTERN DIRECT</t>
+  </si>
+  <si>
     <t>NPS TRUST - A/C KOTAK NPS SANCHAY SCHEME POP</t>
   </si>
   <si>
@@ -640,24 +643,51 @@
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME E - TIER I</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER I</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER I</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I GS</t>
+  </si>
+  <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME A - TIER I</t>
   </si>
   <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME E - TIER II</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER II DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME C - TIER II</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER II DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED SCHEME G - TIER II</t>
   </si>
   <si>
+    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER II DIRECT</t>
+  </si>
+  <si>
     <t>TATA PENSION MANAGEMENT LIMITED TAX SAVER - TIER II</t>
   </si>
   <si>
@@ -667,33 +697,6 @@
     <t>NPS TRUST - A/C TATA PENSION FUND - NPS VATSALYA SCHEME DIRECT</t>
   </si>
   <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I GS</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER I DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME E - TIER II DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME C - TIER II DIRECT</t>
-  </si>
-  <si>
-    <t>NPS TRUST A/C TATA PENSION FUND MANAGEMENT PRIVATE LIMITED SCHEME G - TIER II DIRECT</t>
-  </si>
-  <si>
     <t>NPS TRUST - A/C TATA PENSION FUND - NPS VATSALYA SCHEME POP</t>
   </si>
   <si>
@@ -775,15 +778,15 @@
     <t>NPS TRUST - A/C AXIS NPS SANCHAY SCHEME DIRECT</t>
   </si>
   <si>
+    <t>NPS TRUST A/C DSP PENSION FUND MANAGERS PRIVATE LIMITED SCHEME G - TIER I POP</t>
+  </si>
+  <si>
     <t>NPS TRUST A/C DSP PENSION FUND MANAGERS PRIVATE LIMITED SCHEME E - TIER I POP</t>
   </si>
   <si>
     <t>NPS TRUST A/C DSP PENSION FUND MANAGERS PRIVATE LIMITED SCHEME C - TIER I POP</t>
   </si>
   <si>
-    <t>NPS TRUST A/C DSP PENSION FUND MANAGERS PRIVATE LIMITED SCHEME G - TIER I POP</t>
-  </si>
-  <si>
     <t>NPS TRUST A/C - DSP PENSION FUND MANAGERS PRIVATE LIMITED SCHEME A - TIER I</t>
   </si>
   <si>
@@ -940,102 +943,102 @@
     <t>SM001034</t>
   </si>
   <si>
+    <t>SM002008</t>
+  </si>
+  <si>
+    <t>SM002001</t>
+  </si>
+  <si>
+    <t>SM002002</t>
+  </si>
+  <si>
+    <t>SM002003</t>
+  </si>
+  <si>
+    <t>SM002004</t>
+  </si>
+  <si>
+    <t>SM002005</t>
+  </si>
+  <si>
+    <t>SM002006</t>
+  </si>
+  <si>
+    <t>SM002007</t>
+  </si>
+  <si>
+    <t>SM002009</t>
+  </si>
+  <si>
+    <t>SM002011</t>
+  </si>
+  <si>
+    <t>SM002012</t>
+  </si>
+  <si>
+    <t>SM002014</t>
+  </si>
+  <si>
+    <t>SM002015</t>
+  </si>
+  <si>
+    <t>SM002016</t>
+  </si>
+  <si>
+    <t>SM002017</t>
+  </si>
+  <si>
+    <t>SM002018</t>
+  </si>
+  <si>
+    <t>SM002019</t>
+  </si>
+  <si>
+    <t>SM002020</t>
+  </si>
+  <si>
+    <t>SM002021</t>
+  </si>
+  <si>
+    <t>SM002022</t>
+  </si>
+  <si>
+    <t>SM002023</t>
+  </si>
+  <si>
+    <t>SM002024</t>
+  </si>
+  <si>
+    <t>SM002025</t>
+  </si>
+  <si>
+    <t>SM002026</t>
+  </si>
+  <si>
+    <t>SM002027</t>
+  </si>
+  <si>
+    <t>SM002028</t>
+  </si>
+  <si>
+    <t>SM002029</t>
+  </si>
+  <si>
+    <t>SM002030</t>
+  </si>
+  <si>
+    <t>SM002031</t>
+  </si>
+  <si>
+    <t>SM002032</t>
+  </si>
+  <si>
+    <t>SM002033</t>
+  </si>
+  <si>
     <t>SM002034</t>
   </si>
   <si>
-    <t>SM002001</t>
-  </si>
-  <si>
-    <t>SM002002</t>
-  </si>
-  <si>
-    <t>SM002003</t>
-  </si>
-  <si>
-    <t>SM002004</t>
-  </si>
-  <si>
-    <t>SM002005</t>
-  </si>
-  <si>
-    <t>SM002006</t>
-  </si>
-  <si>
-    <t>SM002007</t>
-  </si>
-  <si>
-    <t>SM002008</t>
-  </si>
-  <si>
-    <t>SM002009</t>
-  </si>
-  <si>
-    <t>SM002011</t>
-  </si>
-  <si>
-    <t>SM002012</t>
-  </si>
-  <si>
-    <t>SM002014</t>
-  </si>
-  <si>
-    <t>SM002015</t>
-  </si>
-  <si>
-    <t>SM002016</t>
-  </si>
-  <si>
-    <t>SM002017</t>
-  </si>
-  <si>
-    <t>SM002018</t>
-  </si>
-  <si>
-    <t>SM002019</t>
-  </si>
-  <si>
-    <t>SM002020</t>
-  </si>
-  <si>
-    <t>SM002021</t>
-  </si>
-  <si>
-    <t>SM002022</t>
-  </si>
-  <si>
-    <t>SM002023</t>
-  </si>
-  <si>
-    <t>SM002024</t>
-  </si>
-  <si>
-    <t>SM002025</t>
-  </si>
-  <si>
-    <t>SM002026</t>
-  </si>
-  <si>
-    <t>SM002027</t>
-  </si>
-  <si>
-    <t>SM002028</t>
-  </si>
-  <si>
-    <t>SM002029</t>
-  </si>
-  <si>
-    <t>SM002030</t>
-  </si>
-  <si>
-    <t>SM002031</t>
-  </si>
-  <si>
-    <t>SM002032</t>
-  </si>
-  <si>
-    <t>SM002033</t>
-  </si>
-  <si>
     <t>SM002035</t>
   </si>
   <si>
@@ -1204,6 +1207,9 @@
     <t>SM005022</t>
   </si>
   <si>
+    <t>SM005023</t>
+  </si>
+  <si>
     <t>SM005024</t>
   </si>
   <si>
@@ -1426,24 +1432,51 @@
     <t>SM011001</t>
   </si>
   <si>
+    <t>SM011011</t>
+  </si>
+  <si>
+    <t>SM011014</t>
+  </si>
+  <si>
     <t>SM011002</t>
   </si>
   <si>
+    <t>SM011012</t>
+  </si>
+  <si>
+    <t>SM011015</t>
+  </si>
+  <si>
     <t>SM011003</t>
   </si>
   <si>
+    <t>SM011013</t>
+  </si>
+  <si>
+    <t>SM011016</t>
+  </si>
+  <si>
     <t>SM011004</t>
   </si>
   <si>
     <t>SM011005</t>
   </si>
   <si>
+    <t>SM011017</t>
+  </si>
+  <si>
     <t>SM011006</t>
   </si>
   <si>
+    <t>SM011018</t>
+  </si>
+  <si>
     <t>SM011007</t>
   </si>
   <si>
+    <t>SM011019</t>
+  </si>
+  <si>
     <t>SM011008</t>
   </si>
   <si>
@@ -1453,33 +1486,6 @@
     <t>SM011010</t>
   </si>
   <si>
-    <t>SM011011</t>
-  </si>
-  <si>
-    <t>SM011012</t>
-  </si>
-  <si>
-    <t>SM011013</t>
-  </si>
-  <si>
-    <t>SM011014</t>
-  </si>
-  <si>
-    <t>SM011015</t>
-  </si>
-  <si>
-    <t>SM011016</t>
-  </si>
-  <si>
-    <t>SM011017</t>
-  </si>
-  <si>
-    <t>SM011018</t>
-  </si>
-  <si>
-    <t>SM011019</t>
-  </si>
-  <si>
     <t>SM011020</t>
   </si>
   <si>
@@ -1561,13 +1567,13 @@
     <t>SM013023</t>
   </si>
   <si>
+    <t>SM014003</t>
+  </si>
+  <si>
     <t>SM014001</t>
   </si>
   <si>
     <t>SM014002</t>
-  </si>
-  <si>
-    <t>SM014003</t>
   </si>
   <si>
     <t>SM014004</t>
@@ -1970,7 +1976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C263"/>
+  <dimension ref="A1:C264"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" style="1" customWidth="1"/>
@@ -1997,7 +2003,7 @@
         <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2008,7 +2014,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2019,7 +2025,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2030,7 +2036,7 @@
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2041,7 +2047,7 @@
         <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2052,7 +2058,7 @@
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2063,7 +2069,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2074,7 +2080,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -2085,7 +2091,7 @@
         <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -2096,7 +2102,7 @@
         <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -2107,7 +2113,7 @@
         <v>23</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -2118,7 +2124,7 @@
         <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -2129,7 +2135,7 @@
         <v>25</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -2140,7 +2146,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2151,7 +2157,7 @@
         <v>27</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -2162,7 +2168,7 @@
         <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2173,7 +2179,7 @@
         <v>29</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -2184,7 +2190,7 @@
         <v>30</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -2195,7 +2201,7 @@
         <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2206,7 +2212,7 @@
         <v>32</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -2217,7 +2223,7 @@
         <v>33</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -2228,7 +2234,7 @@
         <v>34</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -2239,7 +2245,7 @@
         <v>35</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2250,7 +2256,7 @@
         <v>36</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -2261,7 +2267,7 @@
         <v>37</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2272,7 +2278,7 @@
         <v>38</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2283,7 +2289,7 @@
         <v>39</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2294,7 +2300,7 @@
         <v>40</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2305,7 +2311,7 @@
         <v>41</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2316,7 +2322,7 @@
         <v>42</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2327,7 +2333,7 @@
         <v>43</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2338,7 +2344,7 @@
         <v>44</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -2349,7 +2355,7 @@
         <v>45</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -2360,7 +2366,7 @@
         <v>46</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -2371,7 +2377,7 @@
         <v>47</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -2382,7 +2388,7 @@
         <v>48</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -2393,7 +2399,7 @@
         <v>49</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -2404,7 +2410,7 @@
         <v>50</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -2415,7 +2421,7 @@
         <v>51</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -2426,7 +2432,7 @@
         <v>52</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -2437,7 +2443,7 @@
         <v>53</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -2448,7 +2454,7 @@
         <v>54</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -2459,7 +2465,7 @@
         <v>55</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -2470,7 +2476,7 @@
         <v>56</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -2481,7 +2487,7 @@
         <v>57</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -2492,7 +2498,7 @@
         <v>58</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -2503,7 +2509,7 @@
         <v>59</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -2514,7 +2520,7 @@
         <v>60</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -2525,7 +2531,7 @@
         <v>61</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -2536,7 +2542,7 @@
         <v>62</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -2547,7 +2553,7 @@
         <v>63</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -2558,7 +2564,7 @@
         <v>64</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -2569,7 +2575,7 @@
         <v>65</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -2580,7 +2586,7 @@
         <v>66</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -2591,7 +2597,7 @@
         <v>67</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -2602,7 +2608,7 @@
         <v>68</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -2613,7 +2619,7 @@
         <v>69</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -2624,7 +2630,7 @@
         <v>70</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -2635,7 +2641,7 @@
         <v>71</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -2646,7 +2652,7 @@
         <v>72</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -2657,7 +2663,7 @@
         <v>73</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -2668,7 +2674,7 @@
         <v>74</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -2679,7 +2685,7 @@
         <v>75</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -2690,7 +2696,7 @@
         <v>76</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -2701,7 +2707,7 @@
         <v>77</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -2712,7 +2718,7 @@
         <v>78</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -2723,7 +2729,7 @@
         <v>79</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -2734,7 +2740,7 @@
         <v>80</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -2745,7 +2751,7 @@
         <v>81</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -2756,7 +2762,7 @@
         <v>82</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -2767,7 +2773,7 @@
         <v>83</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -2778,7 +2784,7 @@
         <v>84</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -2789,7 +2795,7 @@
         <v>85</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -2800,7 +2806,7 @@
         <v>86</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -2811,7 +2817,7 @@
         <v>87</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -2822,7 +2828,7 @@
         <v>88</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -2833,7 +2839,7 @@
         <v>89</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -2844,7 +2850,7 @@
         <v>90</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -2855,7 +2861,7 @@
         <v>91</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2866,7 +2872,7 @@
         <v>92</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2877,7 +2883,7 @@
         <v>93</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2888,7 +2894,7 @@
         <v>94</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2899,7 +2905,7 @@
         <v>95</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2910,7 +2916,7 @@
         <v>96</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2921,7 +2927,7 @@
         <v>97</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2932,7 +2938,7 @@
         <v>98</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2943,7 +2949,7 @@
         <v>99</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2954,7 +2960,7 @@
         <v>100</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2965,7 +2971,7 @@
         <v>101</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2976,7 +2982,7 @@
         <v>102</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2987,7 +2993,7 @@
         <v>103</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2998,7 +3004,7 @@
         <v>104</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -3009,7 +3015,7 @@
         <v>105</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -3020,7 +3026,7 @@
         <v>106</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -3031,7 +3037,7 @@
         <v>107</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -3042,7 +3048,7 @@
         <v>108</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -3053,7 +3059,7 @@
         <v>109</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -3064,7 +3070,7 @@
         <v>110</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -3075,7 +3081,7 @@
         <v>111</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -3086,7 +3092,7 @@
         <v>112</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -3097,7 +3103,7 @@
         <v>113</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -3108,7 +3114,7 @@
         <v>114</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -3119,7 +3125,7 @@
         <v>115</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -3130,7 +3136,7 @@
         <v>116</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -3141,7 +3147,7 @@
         <v>117</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -3152,7 +3158,7 @@
         <v>118</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -3163,7 +3169,7 @@
         <v>119</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -3174,7 +3180,7 @@
         <v>120</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -3185,7 +3191,7 @@
         <v>121</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -3196,7 +3202,7 @@
         <v>122</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -3207,7 +3213,7 @@
         <v>123</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -3218,7 +3224,7 @@
         <v>124</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -3229,7 +3235,7 @@
         <v>125</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -3240,7 +3246,7 @@
         <v>126</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -3251,7 +3257,7 @@
         <v>127</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -3262,7 +3268,7 @@
         <v>128</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -3273,7 +3279,7 @@
         <v>129</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -3284,7 +3290,7 @@
         <v>130</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -3295,7 +3301,7 @@
         <v>131</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -3306,7 +3312,7 @@
         <v>132</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -3317,7 +3323,7 @@
         <v>133</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -3328,7 +3334,7 @@
         <v>134</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -3339,7 +3345,7 @@
         <v>135</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -3350,18 +3356,18 @@
         <v>136</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>137</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -3372,7 +3378,7 @@
         <v>138</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -3383,7 +3389,7 @@
         <v>139</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -3394,7 +3400,7 @@
         <v>140</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -3405,7 +3411,7 @@
         <v>141</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -3416,7 +3422,7 @@
         <v>142</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -3427,7 +3433,7 @@
         <v>143</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -3438,7 +3444,7 @@
         <v>144</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -3449,7 +3455,7 @@
         <v>145</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -3460,7 +3466,7 @@
         <v>146</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -3471,7 +3477,7 @@
         <v>147</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -3482,7 +3488,7 @@
         <v>148</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -3493,7 +3499,7 @@
         <v>149</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -3504,7 +3510,7 @@
         <v>150</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="140" spans="1:3">
@@ -3515,7 +3521,7 @@
         <v>151</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -3526,7 +3532,7 @@
         <v>152</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="142" spans="1:3">
@@ -3537,7 +3543,7 @@
         <v>153</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -3548,7 +3554,7 @@
         <v>154</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -3559,7 +3565,7 @@
         <v>155</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -3570,7 +3576,7 @@
         <v>156</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -3581,7 +3587,7 @@
         <v>157</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -3592,7 +3598,7 @@
         <v>158</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="148" spans="1:3">
@@ -3603,18 +3609,18 @@
         <v>159</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>160</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="150" spans="1:3">
@@ -3625,7 +3631,7 @@
         <v>161</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -3636,7 +3642,7 @@
         <v>162</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -3647,7 +3653,7 @@
         <v>163</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -3658,7 +3664,7 @@
         <v>164</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -3669,7 +3675,7 @@
         <v>165</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="155" spans="1:3">
@@ -3680,7 +3686,7 @@
         <v>166</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -3691,7 +3697,7 @@
         <v>167</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="157" spans="1:3">
@@ -3702,7 +3708,7 @@
         <v>168</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -3713,7 +3719,7 @@
         <v>169</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -3724,7 +3730,7 @@
         <v>170</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="160" spans="1:3">
@@ -3735,7 +3741,7 @@
         <v>171</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -3746,7 +3752,7 @@
         <v>172</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="162" spans="1:3">
@@ -3757,7 +3763,7 @@
         <v>173</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -3768,7 +3774,7 @@
         <v>174</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -3779,7 +3785,7 @@
         <v>175</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -3790,7 +3796,7 @@
         <v>176</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="166" spans="1:3">
@@ -3801,7 +3807,7 @@
         <v>177</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -3812,7 +3818,7 @@
         <v>178</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="168" spans="1:3">
@@ -3823,7 +3829,7 @@
         <v>179</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="169" spans="1:3">
@@ -3834,7 +3840,7 @@
         <v>180</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -3845,7 +3851,7 @@
         <v>181</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -3856,7 +3862,7 @@
         <v>182</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -3867,18 +3873,18 @@
         <v>183</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B173" s="1" t="s">
         <v>184</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="174" spans="1:3">
@@ -3889,7 +3895,7 @@
         <v>185</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -3900,7 +3906,7 @@
         <v>186</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -3911,7 +3917,7 @@
         <v>187</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -3922,7 +3928,7 @@
         <v>188</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -3933,7 +3939,7 @@
         <v>189</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -3944,7 +3950,7 @@
         <v>190</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -3955,7 +3961,7 @@
         <v>191</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -3966,7 +3972,7 @@
         <v>192</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -3977,7 +3983,7 @@
         <v>193</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -3988,7 +3994,7 @@
         <v>194</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -3999,7 +4005,7 @@
         <v>195</v>
       </c>
       <c r="C184" s="1" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -4010,7 +4016,7 @@
         <v>196</v>
       </c>
       <c r="C185" s="1" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -4021,7 +4027,7 @@
         <v>197</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -4032,7 +4038,7 @@
         <v>198</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -4043,7 +4049,7 @@
         <v>199</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="189" spans="1:3">
@@ -4054,7 +4060,7 @@
         <v>200</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="190" spans="1:3">
@@ -4065,7 +4071,7 @@
         <v>201</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -4076,7 +4082,7 @@
         <v>202</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="192" spans="1:3">
@@ -4087,7 +4093,7 @@
         <v>203</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="193" spans="1:3">
@@ -4098,7 +4104,7 @@
         <v>204</v>
       </c>
       <c r="C193" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -4109,7 +4115,7 @@
         <v>205</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -4120,18 +4126,18 @@
         <v>206</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>207</v>
       </c>
       <c r="C196" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -4142,7 +4148,7 @@
         <v>208</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -4153,7 +4159,7 @@
         <v>209</v>
       </c>
       <c r="C198" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -4164,7 +4170,7 @@
         <v>210</v>
       </c>
       <c r="C199" s="1" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="200" spans="1:3">
@@ -4175,7 +4181,7 @@
         <v>211</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -4186,7 +4192,7 @@
         <v>212</v>
       </c>
       <c r="C201" s="1" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -4197,7 +4203,7 @@
         <v>213</v>
       </c>
       <c r="C202" s="1" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -4208,7 +4214,7 @@
         <v>214</v>
       </c>
       <c r="C203" s="1" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -4219,7 +4225,7 @@
         <v>215</v>
       </c>
       <c r="C204" s="1" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -4230,7 +4236,7 @@
         <v>216</v>
       </c>
       <c r="C205" s="1" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -4241,7 +4247,7 @@
         <v>217</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -4252,7 +4258,7 @@
         <v>218</v>
       </c>
       <c r="C207" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -4263,7 +4269,7 @@
         <v>219</v>
       </c>
       <c r="C208" s="1" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="209" spans="1:3">
@@ -4274,7 +4280,7 @@
         <v>220</v>
       </c>
       <c r="C209" s="1" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -4285,7 +4291,7 @@
         <v>221</v>
       </c>
       <c r="C210" s="1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="211" spans="1:3">
@@ -4296,7 +4302,7 @@
         <v>222</v>
       </c>
       <c r="C211" s="1" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="212" spans="1:3">
@@ -4307,7 +4313,7 @@
         <v>223</v>
       </c>
       <c r="C212" s="1" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="213" spans="1:3">
@@ -4318,7 +4324,7 @@
         <v>224</v>
       </c>
       <c r="C213" s="1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -4329,7 +4335,7 @@
         <v>225</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="215" spans="1:3">
@@ -4340,7 +4346,7 @@
         <v>226</v>
       </c>
       <c r="C215" s="1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="216" spans="1:3">
@@ -4351,7 +4357,7 @@
         <v>227</v>
       </c>
       <c r="C216" s="1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -4362,7 +4368,7 @@
         <v>228</v>
       </c>
       <c r="C217" s="1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -4373,18 +4379,18 @@
         <v>229</v>
       </c>
       <c r="C218" s="1" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>230</v>
       </c>
       <c r="C219" s="1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -4395,7 +4401,7 @@
         <v>231</v>
       </c>
       <c r="C220" s="1" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -4406,7 +4412,7 @@
         <v>232</v>
       </c>
       <c r="C221" s="1" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -4417,7 +4423,7 @@
         <v>233</v>
       </c>
       <c r="C222" s="1" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -4428,7 +4434,7 @@
         <v>234</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -4439,7 +4445,7 @@
         <v>235</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -4450,7 +4456,7 @@
         <v>236</v>
       </c>
       <c r="C225" s="1" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -4461,7 +4467,7 @@
         <v>237</v>
       </c>
       <c r="C226" s="1" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="227" spans="1:3">
@@ -4472,7 +4478,7 @@
         <v>238</v>
       </c>
       <c r="C227" s="1" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -4483,7 +4489,7 @@
         <v>239</v>
       </c>
       <c r="C228" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="229" spans="1:3">
@@ -4494,7 +4500,7 @@
         <v>240</v>
       </c>
       <c r="C229" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -4505,7 +4511,7 @@
         <v>241</v>
       </c>
       <c r="C230" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -4516,7 +4522,7 @@
         <v>242</v>
       </c>
       <c r="C231" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -4527,7 +4533,7 @@
         <v>243</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -4538,7 +4544,7 @@
         <v>244</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -4549,7 +4555,7 @@
         <v>245</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -4560,7 +4566,7 @@
         <v>246</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -4571,7 +4577,7 @@
         <v>247</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -4582,7 +4588,7 @@
         <v>248</v>
       </c>
       <c r="C237" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="238" spans="1:3">
@@ -4593,7 +4599,7 @@
         <v>249</v>
       </c>
       <c r="C238" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="239" spans="1:3">
@@ -4604,7 +4610,7 @@
         <v>250</v>
       </c>
       <c r="C239" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -4615,7 +4621,7 @@
         <v>251</v>
       </c>
       <c r="C240" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -4626,18 +4632,18 @@
         <v>252</v>
       </c>
       <c r="C241" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>253</v>
       </c>
       <c r="C242" s="1" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -4648,7 +4654,7 @@
         <v>254</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -4659,7 +4665,7 @@
         <v>255</v>
       </c>
       <c r="C244" s="1" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -4670,7 +4676,7 @@
         <v>256</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -4681,7 +4687,7 @@
         <v>257</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -4692,7 +4698,7 @@
         <v>258</v>
       </c>
       <c r="C247" s="1" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -4703,7 +4709,7 @@
         <v>259</v>
       </c>
       <c r="C248" s="1" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -4714,7 +4720,7 @@
         <v>260</v>
       </c>
       <c r="C249" s="1" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
     </row>
     <row r="250" spans="1:3">
@@ -4725,7 +4731,7 @@
         <v>261</v>
       </c>
       <c r="C250" s="1" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -4736,7 +4742,7 @@
         <v>262</v>
       </c>
       <c r="C251" s="1" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="252" spans="1:3">
@@ -4747,7 +4753,7 @@
         <v>263</v>
       </c>
       <c r="C252" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="253" spans="1:3">
@@ -4758,7 +4764,7 @@
         <v>264</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="254" spans="1:3">
@@ -4769,7 +4775,7 @@
         <v>265</v>
       </c>
       <c r="C254" s="1" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
     </row>
     <row r="255" spans="1:3">
@@ -4780,7 +4786,7 @@
         <v>266</v>
       </c>
       <c r="C255" s="1" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="256" spans="1:3">
@@ -4791,7 +4797,7 @@
         <v>267</v>
       </c>
       <c r="C256" s="1" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="257" spans="1:3">
@@ -4802,7 +4808,7 @@
         <v>268</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="258" spans="1:3">
@@ -4813,7 +4819,7 @@
         <v>269</v>
       </c>
       <c r="C258" s="1" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="259" spans="1:3">
@@ -4824,7 +4830,7 @@
         <v>270</v>
       </c>
       <c r="C259" s="1" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="260" spans="1:3">
@@ -4835,7 +4841,7 @@
         <v>271</v>
       </c>
       <c r="C260" s="1" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="261" spans="1:3">
@@ -4846,7 +4852,7 @@
         <v>272</v>
       </c>
       <c r="C261" s="1" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="262" spans="1:3">
@@ -4857,7 +4863,7 @@
         <v>273</v>
       </c>
       <c r="C262" s="1" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
     </row>
     <row r="263" spans="1:3">
@@ -4868,7 +4874,18 @@
         <v>274</v>
       </c>
       <c r="C263" s="1" t="s">
-        <v>536</v>
+        <v>537</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3">
+      <c r="A264" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C264" s="1" t="s">
+        <v>538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>